<commit_message>
fix(units): release corrected unit contracts
- prioritize percent for AID/ATTD GE coefficients
- correct the synthetic SID percentage example
- preserve released model assets and results
</commit_message>
<xml_diff>
--- a/templates/feed_ingredient_contribution_template.xlsx
+++ b/templates/feed_ingredient_contribution_template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions_说明" sheetId="1" r:id="R4f8f17fe3271483b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Article Metadata" sheetId="2" r:id="R29d5dfaac53d46d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingredient Data" sheetId="3" r:id="R71407da3ef2b4c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions_说明" sheetId="1" r:id="Re6446edee8424e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Article Metadata" sheetId="2" r:id="R731abc7da76a418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ingredient Data" sheetId="3" r:id="R7c7d347f96044a25"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -465,10 +465,10 @@
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="64" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1437,16 +1437,16 @@
         <x:v>Unit</x:v>
       </x:c>
       <x:c r="E38" s="35" t="str">
-        <x:v>来源明确单位优先；未知时留空待核对 / Explicit source unit has priority; blank triggers review</x:v>
+        <x:v>来源明确单位优先；能量缺失单位时界面建议可编辑MJ/kg，不换算原始值 / Explicit source unit has priority; blank energy receives an editable MJ/kg suggestion without rescaling the value</x:v>
       </x:c>
       <x:c r="F38" s="35" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="G38" s="35" t="str">
-        <x:v>e.g. %, g/kg, mg/kg, MJ/kg, kJ/kg</x:v>
+        <x:v>e.g. %, g/kg, mg/kg, MJ/kg, kJ/kg, kcal/kg</x:v>
       </x:c>
       <x:c r="H38" s="35" t="str">
-        <x:v>metric-specific</x:v>
+        <x:v>energy: MJ/kg; composition/digestibility: %</x:v>
       </x:c>
       <x:c r="I38" s="36" t="str">
         <x:v>MJ/kg</x:v>

</xml_diff>